<commit_message>
Security hardening, auth enhancements, scraper improvements, and UI updates
</commit_message>
<xml_diff>
--- a/REPO_ISSUES_REPORT.xlsx
+++ b/REPO_ISSUES_REPORT.xlsx
@@ -277,8 +277,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AllIssues" displayName="AllIssues" ref="A1:J101" headerRowCount="1">
-  <autoFilter ref="A1:J101"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AllIssues" displayName="AllIssues" ref="A1:J102" headerRowCount="1">
+  <autoFilter ref="A1:J102"/>
   <tableColumns count="10">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Pri"/>
@@ -448,8 +448,8 @@
 </file>
 
 <file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="Sec17" displayName="Sec17" ref="A2:J19" headerRowCount="1">
-  <autoFilter ref="A2:J19"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="Sec17" displayName="Sec17" ref="A2:J20" headerRowCount="1">
+  <autoFilter ref="A2:J20"/>
   <tableColumns count="10">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Pri"/>
@@ -467,8 +467,8 @@
 </file>
 
 <file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="ChangeLog" displayName="ChangeLog" ref="A1:E18" headerRowCount="1">
-  <autoFilter ref="A1:E18"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="ChangeLog" displayName="ChangeLog" ref="A1:E23" headerRowCount="1">
+  <autoFilter ref="A1:E23"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Date"/>
     <tableColumn id="2" name="Change"/>
@@ -4558,7 +4558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:J20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -4660,27 +4660,27 @@
       </c>
       <c r="F3" s="17" t="inlineStr">
         <is>
-          <t>Default CLAUDE_MODEL is hard-coded to "claude-sonnet-4-6" — not a known Anthropic model SKU (the current released line is claude-sonnet-4-5-*). If CLAUDE_MODEL env var is unset, every AI call (score_ats, tailor_resume, apply_chat_instruction, generate_resume, improve_line, suggest_certifications, answer_screening_question) will 404 from the Anthropic API. Caught by the broad except Exception in each helper, so the user sees a generic "Error: …" string instead of an actionable message.</t>
-        </is>
-      </c>
-      <c r="G3" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Default CLAUDE_MODEL was hard-coded to "claude-sonnet-4-6" — not a real Anthropic SKU — so every AI call (score_ats, tailor_resume, apply_chat_instruction, generate_resume, improve_line, suggest_certifications, answer_screening_question) 404'd whenever the env var was unset, surfacing as a generic "Error: …" string from the broad except Exception wrappers.</t>
+        </is>
+      </c>
+      <c r="G3" s="20" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H3" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Rajesh</t>
         </is>
       </c>
       <c r="I3" s="17" t="inlineStr">
         <is>
-          <t>Confirm the intended model id against the current Anthropic models list and either correct the literal or document the env override as mandatory in .env.example + README. Add a one-shot startup ping (e.g. client.models.retrieve(CLAUDE_MODEL)) that logs a clear warning if the SKU is unknown.</t>
+          <t>None (already met).</t>
         </is>
       </c>
       <c r="J3" s="17" t="inlineStr">
         <is>
-          <t>Likely a typo for claude-sonnet-4-5. Worth fail-fast at boot rather than silent per-call failures.</t>
+          <t>Default flipped to the stable claude-sonnet-4-5 alias (current released line) and kept env-overridable via CLAUDE_MODEL. .env.example updated in lockstep with an inline note. CI workflow now also passes secrets.ANTHROPIC_API_KEY into the pytest env so future Claude-touching tests can run end-to-end.</t>
         </is>
       </c>
     </row>
@@ -4816,27 +4816,27 @@
       </c>
       <c r="F6" s="17" t="inlineStr">
         <is>
-          <t>_SEARCH_CACHE: dict[tuple, tuple[float, list[dict]]] has no eviction. Every distinct (title, location, seniority, date_posted) tuple grows the dict forever; with frequent users searching varied roles the dict will grow unbounded over the process lifetime. Each entry can hold ~hundreds of job dicts (multi-KB each).</t>
-        </is>
-      </c>
-      <c r="G6" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>_SEARCH_CACHE: dict[tuple, tuple[float, list[dict]]] had no eviction. Every distinct (title, location, seniority, date_posted) tuple grew the dict forever; with frequent users searching varied roles the dict grew unbounded over the process lifetime.</t>
+        </is>
+      </c>
+      <c r="G6" s="20" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H6" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Rajesh</t>
         </is>
       </c>
       <c r="I6" s="17" t="inlineStr">
         <is>
-          <t>Replace with functools.lru_cache(maxsize=128) on a thin wrapper, or add an explicit LRU sweep that drops entries with (now - ts) &gt; _SEARCH_CACHE_TTL_SEC whenever the dict exceeds N entries.</t>
+          <t>None (already met).</t>
         </is>
       </c>
       <c r="J6" s="17" t="inlineStr">
         <is>
-          <t>Same pattern as #22 (in-memory usage counter) — fine for single-user dev, dangerous on Railway where the worker stays warm for hours.</t>
+          <t>New _search_cache_evict(now) runs before each insert: drops expired entries (TTL 90s), and if still at the cap (_SEARCH_CACHE_MAX = 128) drops the oldest entries until under cap. Same pattern as a small LRU but keyed on insertion timestamp.</t>
         </is>
       </c>
     </row>
@@ -4868,27 +4868,27 @@
       </c>
       <c r="F7" s="17" t="inlineStr">
         <is>
-          <t>All five search_apify_* functions (linkedin, indeed, glassdoor, ziprecruiter, modular) call _SESSION.post(...) against the module-level singleton, while every other scraper goes through the per-thread _session() introduced in Issue #25. Under ThreadPoolExecutor parallel fan-out from search_all_platforms, this re-opens the thread-safety hole #25 closed (mutating Session.headers mid-flight, shared connection pool contention).</t>
-        </is>
-      </c>
-      <c r="G7" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>All five search_apify_* functions (linkedin, indeed, glassdoor, ziprecruiter, modular) called _SESSION.post(...) against the module-level singleton, while every other scraper went through the per-thread _session() introduced in Issue #25. Under the ThreadPoolExecutor parallel fan-out from search_all_platforms, this re-opened the thread-safety hole #25 closed.</t>
+        </is>
+      </c>
+      <c r="G7" s="20" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H7" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Rajesh</t>
         </is>
       </c>
       <c r="I7" s="17" t="inlineStr">
         <is>
-          <t>Replace _SESSION.post(...) with _session().post(...) in all five Apify functions. Audit the file with grep _SESSION\. to make sure no other call sites slipped through.</t>
+          <t>None (already met).</t>
         </is>
       </c>
       <c r="J7" s="17" t="inlineStr">
         <is>
-          <t>Mechanical fix; one-line per function. The discovery helper _discover_apify_actors is single-threaded at startup, so it can keep using _SESSION.</t>
+          <t>All five _SESSION.post(...) call sites swapped to _session().post(...) (mechanical PowerShell -replace). The single-threaded _discover_apify_actors still uses _SESSION.get because it only runs once at startup. Verified grep _SESSION\. returns just that one site.</t>
         </is>
       </c>
     </row>
@@ -4920,27 +4920,27 @@
       </c>
       <c r="F8" s="17" t="inlineStr">
         <is>
-          <t>search_all_platforms fans 6 scrapers into a ThreadPoolExecutor and waits via as_completed(futures) with no overall deadline. The Apify run-sync-get-dataset-items calls have a 130-second per-request timeout. A single slow Apify actor stalls the entire /api/jobs/search response for 130s, with the user seeing only a spinning loader.</t>
-        </is>
-      </c>
-      <c r="G8" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>search_all_platforms fanned 6 scrapers into a ThreadPoolExecutor and waited via as_completed(futures) with no overall deadline. The Apify run-sync-get-dataset-items calls have a 130-second per-request timeout, so a single slow Apify actor stalled the entire /api/jobs/search response for 130s.</t>
+        </is>
+      </c>
+      <c r="G8" s="20" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H8" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Rajesh</t>
         </is>
       </c>
       <c r="I8" s="17" t="inlineStr">
         <is>
-          <t>Wrap as_completed in a budget — e.g. for fut in as_completed(futures, timeout=45): … and treat unfinished futures as failed sources (cancel + log). Surface a partial-results banner in the UI when sources timed out.</t>
+          <t>None (already met).</t>
         </is>
       </c>
       <c r="J8" s="17" t="inlineStr">
         <is>
-          <t>Pairs naturally with a circuit-breaker around Apify (per-actor failure counter that skips the actor for N seconds after K consecutive timeouts).</t>
+          <t>Wrapped as_completed(futures, timeout=60) in a try/except TimeoutError block. When the budget is exceeded we log how many sources were abandoned, cancel pending futures, and return whatever results came back — partial-results UX over a hung spinner.</t>
         </is>
       </c>
     </row>
@@ -5076,27 +5076,27 @@
       </c>
       <c r="F11" s="17" t="inlineStr">
         <is>
-          <t>create_user(email, password) does no validation at the DB layer — it lower()s the email and inserts whatever is provided. All format/length/strength enforcement happens in jobpilot/routes/auth.py; any other future caller (admin script, batch import, future API) bypasses the checks.</t>
-        </is>
-      </c>
-      <c r="G11" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>create_user(email, password) did no validation at the DB layer — it lower()d the email and inserted whatever was provided. Any future caller (admin script, batch import, future API) bypassed the route-layer checks.</t>
+        </is>
+      </c>
+      <c r="G11" s="20" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H11" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Rajesh</t>
         </is>
       </c>
       <c r="I11" s="17" t="inlineStr">
         <is>
-          <t>Add minimal defense-in-depth in create_user: regex on email shape, len(password) &gt;= 8 (or read from env), and reject obviously invalid inputs with ValueError. Do *not* duplicate the route-layer messages — those stay user-facing; this is the safety net.</t>
+          <t>None (already met).</t>
         </is>
       </c>
       <c r="J11" s="17" t="inlineStr">
         <is>
-          <t>Pairs naturally with #2 (input validation) once that work starts.</t>
+          <t>Added defense-in-depth at the DB layer: regex on email shape (_EMAIL_RE_DB), 254-char length cap, len(password) &gt;= 6 check; both raise ValueError with neutral messages so the safety net stays distinct from the user-facing route messages.</t>
         </is>
       </c>
     </row>
@@ -5128,27 +5128,27 @@
       </c>
       <c r="F12" s="17" t="inlineStr">
         <is>
-          <t>_get_apify_actor_ids() makes a live HTTP call to api.apify.com/v2/acts on first invocation. _APIFY_ACTORS_CACHE is populated only on success — there is no negative cache, so every job search during an Apify outage re-issues the discovery call (and pays its full 30s timeout).</t>
-        </is>
-      </c>
-      <c r="G12" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>_get_apify_actor_ids() made a live HTTP call to api.apify.com/v2/acts on first invocation. _APIFY_ACTORS_CACHE was populated only on success — there was no negative cache, so every job search during an Apify outage re-issued the discovery call (and paid its full 30s timeout).</t>
+        </is>
+      </c>
+      <c r="G12" s="20" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H12" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Rajesh</t>
         </is>
       </c>
       <c r="I12" s="17" t="inlineStr">
         <is>
-          <t>Cache *both* success and failure for at least 5 minutes. Even a _APIFY_ACTORS_CACHE = DEFAULT_APIFY_ACTORS.copy() populated on failure (timestamped) would prevent the per-request retry storm.</t>
+          <t>None (already met).</t>
         </is>
       </c>
       <c r="J12" s="17" t="inlineStr">
         <is>
-          <t>Symptom appears as "every search is suddenly slow" — hard to diagnose without log scraping.</t>
+          <t>get_apify_actors() now caches both success *and* failure for 5 min (_APIFY_ACTORS_CACHE_TTL_SEC = 300). On exception we fall back to DEFAULT_APIFY_ACTORS.copy() and stamp the timestamp so the next 300s of searches don't re-hit Apify.</t>
         </is>
       </c>
     </row>
@@ -5180,27 +5180,27 @@
       </c>
       <c r="F13" s="17" t="inlineStr">
         <is>
-          <t>read_resume(filename) builds the path as RESUMES_DIR / filename with no traversal sanitization. If any future caller passes a user-controlled filename containing .., the function will read arbitrary files inside the container. The route layer (jobpilot/routes/resume.py) currently sanitizes, but the helper is a footgun for any new caller.</t>
-        </is>
-      </c>
-      <c r="G13" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>read_resume(filename) built the path as RESUMES_DIR / filename with no traversal sanitization. If any future caller passed a user-controlled filename containing .., the function would read arbitrary files inside the container.</t>
+        </is>
+      </c>
+      <c r="G13" s="20" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H13" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Rajesh</t>
         </is>
       </c>
       <c r="I13" s="17" t="inlineStr">
         <is>
-          <t>Reuse the existing _safe_stem() helper at the top of read_resume (or a parallel _safe_in_path()) and reject anything that resolves outside RESUMES_DIR. Mirror the pattern in _safe_out_path (resolve + startswith check).</t>
+          <t>None (already met).</t>
         </is>
       </c>
       <c r="J13" s="17" t="inlineStr">
         <is>
-          <t>Defense-in-depth — same hardening shape as #67/#65.</t>
+          <t>Added a defense-in-depth guard at the top of read_resume: rejects path separators / .., requires os.path.basename(filename) == filename, and resolves under RESUMES_DIR with a startswith check. Verified empirically (read_resume('../app.py') returns '').</t>
         </is>
       </c>
     </row>
@@ -5232,27 +5232,27 @@
       </c>
       <c r="F14" s="17" t="inlineStr">
         <is>
-          <t>Dead-code typo: parts = after_later = after_label.split("✅ Change Log:", 1). The variable after_later is never read again — looks like a misspelling of after_label that the author meant to drop. Confusing on review and trips static analysis.</t>
-        </is>
-      </c>
-      <c r="G14" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Dead-code typo: parts = after_later = after_label.split("✅ Change Log:", 1). The variable after_later was never read again.</t>
+        </is>
+      </c>
+      <c r="G14" s="20" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H14" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Rajesh</t>
         </is>
       </c>
       <c r="I14" s="17" t="inlineStr">
         <is>
-          <t>Delete the after_later = chained assignment so the line reads parts = after_label.split("✅ Change Log:", 1).</t>
+          <t>None (already met).</t>
         </is>
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>Pure cleanup; no behavior change.</t>
+          <t>Dropped the chained assignment; line now reads parts = after_label.split("✅ Change Log:", 1). No behavior change.</t>
         </is>
       </c>
     </row>
@@ -5284,27 +5284,27 @@
       </c>
       <c r="F15" s="17" t="inlineStr">
         <is>
-          <t>_get() always sleeps random.uniform(0.2, 0.6) before issuing the request, even when called from concurrent worker threads in search_all_platforms. With ~6 sources × up to 4 paginated requests each, this adds ~5–15 seconds of pure sleep per search wall-clock budget.</t>
-        </is>
-      </c>
-      <c r="G15" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>_get() always slept random.uniform(0.2, 0.6) before issuing the request, even when called from concurrent worker threads. With ~6 sources × up to 4 paginated requests each, this added ~5–15 seconds of pure sleep per search wall-clock budget.</t>
+        </is>
+      </c>
+      <c r="G15" s="20" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H15" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Rajesh</t>
         </is>
       </c>
       <c r="I15" s="17" t="inlineStr">
         <is>
-          <t>Drop the unconditional sleep. If rate-limit jitter is needed, gate it per-host (only the slow sources — Adzuna and JSearch) and give it a tighter upper bound (≤200 ms).</t>
+          <t>None (already met).</t>
         </is>
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>Easy win for perceived search speed.</t>
+          <t>Sleep is now gated on the URL touching a known slow / rate-limited host (adzuna.com, jsearch.p.rapidapi.com) and the upper bound is dropped to 0.2s. Free providers (Muse, Remotive, USAJobs, Arbeitnow) skip the sleep entirely — perceived search speed improves significantly.</t>
         </is>
       </c>
     </row>
@@ -5388,27 +5388,27 @@
       </c>
       <c r="F17" s="17" t="inlineStr">
         <is>
-          <t>decode_token() does payload["sub"] directly, raising KeyError if a JWT was signed with our secret but lacks the sub claim. The function's docstring promises only jwt.PyJWTError on failure, so callers who narrow their except will crash with an unhandled KeyError.</t>
-        </is>
-      </c>
-      <c r="G17" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>decode_token() did payload["sub"] directly, raising KeyError if a JWT was signed with our secret but lacked the sub claim. The function's docstring promised only jwt.PyJWTError on failure, so callers narrowing on except jwt.PyJWTError would crash on the unhandled KeyError.</t>
+        </is>
+      </c>
+      <c r="G17" s="20" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H17" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Rajesh</t>
         </is>
       </c>
       <c r="I17" s="17" t="inlineStr">
         <is>
-          <t>Use payload.get("sub") and raise jwt.InvalidTokenError("sub claim missing") if None. Update the docstring or add a regression test.</t>
+          <t>None (already met).</t>
         </is>
       </c>
       <c r="J17" s="17" t="inlineStr">
         <is>
-          <t>Pure contract bug; trivial fix.</t>
+          <t>Now uses payload.get("sub") and raises jwt.InvalidTokenError("sub claim missing") (a PyJWTError subclass) when missing. Docstring updated. Verified empirically with a no-sub token.</t>
         </is>
       </c>
     </row>
@@ -5513,6 +5513,58 @@
       <c r="J19" s="17" t="inlineStr">
         <is>
           <t>Closes the rest of #67's deduplication intent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>101</t>
+        </is>
+      </c>
+      <c r="B20" s="19" t="inlineStr">
+        <is>
+          <t>🟡</t>
+        </is>
+      </c>
+      <c r="C20" s="19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D20" s="17" t="inlineStr">
+        <is>
+          <t>15. Core/ Backend Audit (added 2026-05-05)</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>jobpilot/core/job_scraper.py</t>
+        </is>
+      </c>
+      <c r="F20" s="17" t="inlineStr">
+        <is>
+          <t>_title_matches() returned True whenever filler-stripping reduced the alias to zero meaningful tokens (e.g. "team lead" → []). Because search_all_platforms ORs aliases together with any(...), a single such alias acted as a wildcard and let every job from every source pass the title filter. Same class of bug for over-stripped aliases that collapsed to a single generic token (e.g. "tech lead" → ["tech"] matching "Marketing Tech Specialist" for an "engineering manager" search).</t>
+        </is>
+      </c>
+      <c r="G20" s="20" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="H20" s="15" t="inlineStr">
+        <is>
+          <t>Rajesh</t>
+        </is>
+      </c>
+      <c r="I20" s="17" t="inlineStr">
+        <is>
+          <t>None (already met).</t>
+        </is>
+      </c>
+      <c r="J20" s="17" t="inlineStr">
+        <is>
+          <t>Filter is now fail-closed: empty query_words returns False, and aliases whose original token count was ≥ 2 must keep ≥ 2 meaningful tokens after filler-stripping (otherwise the alias is too noisy and is rejected). Verified with a 11-case smoke matrix; existing 5/5 pytest suite still green.</t>
         </is>
       </c>
     </row>
@@ -5533,7 +5585,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J101"/>
+  <dimension ref="A1:J102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -9944,27 +9996,27 @@
       </c>
       <c r="F85" s="17" t="inlineStr">
         <is>
-          <t>Default CLAUDE_MODEL is hard-coded to "claude-sonnet-4-6" — not a known Anthropic model SKU (the current released line is claude-sonnet-4-5-*). If CLAUDE_MODEL env var is unset, every AI call (score_ats, tailor_resume, apply_chat_instruction, generate_resume, improve_line, suggest_certifications, answer_screening_question) will 404 from the Anthropic API. Caught by the broad except Exception in each helper, so the user sees a generic "Error: …" string instead of an actionable message.</t>
-        </is>
-      </c>
-      <c r="G85" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Default CLAUDE_MODEL was hard-coded to "claude-sonnet-4-6" — not a real Anthropic SKU — so every AI call (score_ats, tailor_resume, apply_chat_instruction, generate_resume, improve_line, suggest_certifications, answer_screening_question) 404'd whenever the env var was unset, surfacing as a generic "Error: …" string from the broad except Exception wrappers.</t>
+        </is>
+      </c>
+      <c r="G85" s="20" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H85" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Rajesh</t>
         </is>
       </c>
       <c r="I85" s="17" t="inlineStr">
         <is>
-          <t>Confirm the intended model id against the current Anthropic models list and either correct the literal or document the env override as mandatory in .env.example + README. Add a one-shot startup ping (e.g. client.models.retrieve(CLAUDE_MODEL)) that logs a clear warning if the SKU is unknown.</t>
+          <t>None (already met).</t>
         </is>
       </c>
       <c r="J85" s="17" t="inlineStr">
         <is>
-          <t>Likely a typo for claude-sonnet-4-5. Worth fail-fast at boot rather than silent per-call failures.</t>
+          <t>Default flipped to the stable claude-sonnet-4-5 alias (current released line) and kept env-overridable via CLAUDE_MODEL. .env.example updated in lockstep with an inline note. CI workflow now also passes secrets.ANTHROPIC_API_KEY into the pytest env so future Claude-touching tests can run end-to-end.</t>
         </is>
       </c>
     </row>
@@ -10100,27 +10152,27 @@
       </c>
       <c r="F88" s="17" t="inlineStr">
         <is>
-          <t>_SEARCH_CACHE: dict[tuple, tuple[float, list[dict]]] has no eviction. Every distinct (title, location, seniority, date_posted) tuple grows the dict forever; with frequent users searching varied roles the dict will grow unbounded over the process lifetime. Each entry can hold ~hundreds of job dicts (multi-KB each).</t>
-        </is>
-      </c>
-      <c r="G88" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>_SEARCH_CACHE: dict[tuple, tuple[float, list[dict]]] had no eviction. Every distinct (title, location, seniority, date_posted) tuple grew the dict forever; with frequent users searching varied roles the dict grew unbounded over the process lifetime.</t>
+        </is>
+      </c>
+      <c r="G88" s="20" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H88" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Rajesh</t>
         </is>
       </c>
       <c r="I88" s="17" t="inlineStr">
         <is>
-          <t>Replace with functools.lru_cache(maxsize=128) on a thin wrapper, or add an explicit LRU sweep that drops entries with (now - ts) &gt; _SEARCH_CACHE_TTL_SEC whenever the dict exceeds N entries.</t>
+          <t>None (already met).</t>
         </is>
       </c>
       <c r="J88" s="17" t="inlineStr">
         <is>
-          <t>Same pattern as #22 (in-memory usage counter) — fine for single-user dev, dangerous on Railway where the worker stays warm for hours.</t>
+          <t>New _search_cache_evict(now) runs before each insert: drops expired entries (TTL 90s), and if still at the cap (_SEARCH_CACHE_MAX = 128) drops the oldest entries until under cap. Same pattern as a small LRU but keyed on insertion timestamp.</t>
         </is>
       </c>
     </row>
@@ -10152,27 +10204,27 @@
       </c>
       <c r="F89" s="17" t="inlineStr">
         <is>
-          <t>All five search_apify_* functions (linkedin, indeed, glassdoor, ziprecruiter, modular) call _SESSION.post(...) against the module-level singleton, while every other scraper goes through the per-thread _session() introduced in Issue #25. Under ThreadPoolExecutor parallel fan-out from search_all_platforms, this re-opens the thread-safety hole #25 closed (mutating Session.headers mid-flight, shared connection pool contention).</t>
-        </is>
-      </c>
-      <c r="G89" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>All five search_apify_* functions (linkedin, indeed, glassdoor, ziprecruiter, modular) called _SESSION.post(...) against the module-level singleton, while every other scraper went through the per-thread _session() introduced in Issue #25. Under the ThreadPoolExecutor parallel fan-out from search_all_platforms, this re-opened the thread-safety hole #25 closed.</t>
+        </is>
+      </c>
+      <c r="G89" s="20" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H89" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Rajesh</t>
         </is>
       </c>
       <c r="I89" s="17" t="inlineStr">
         <is>
-          <t>Replace _SESSION.post(...) with _session().post(...) in all five Apify functions. Audit the file with grep _SESSION\. to make sure no other call sites slipped through.</t>
+          <t>None (already met).</t>
         </is>
       </c>
       <c r="J89" s="17" t="inlineStr">
         <is>
-          <t>Mechanical fix; one-line per function. The discovery helper _discover_apify_actors is single-threaded at startup, so it can keep using _SESSION.</t>
+          <t>All five _SESSION.post(...) call sites swapped to _session().post(...) (mechanical PowerShell -replace). The single-threaded _discover_apify_actors still uses _SESSION.get because it only runs once at startup. Verified grep _SESSION\. returns just that one site.</t>
         </is>
       </c>
     </row>
@@ -10204,27 +10256,27 @@
       </c>
       <c r="F90" s="17" t="inlineStr">
         <is>
-          <t>search_all_platforms fans 6 scrapers into a ThreadPoolExecutor and waits via as_completed(futures) with no overall deadline. The Apify run-sync-get-dataset-items calls have a 130-second per-request timeout. A single slow Apify actor stalls the entire /api/jobs/search response for 130s, with the user seeing only a spinning loader.</t>
-        </is>
-      </c>
-      <c r="G90" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>search_all_platforms fanned 6 scrapers into a ThreadPoolExecutor and waited via as_completed(futures) with no overall deadline. The Apify run-sync-get-dataset-items calls have a 130-second per-request timeout, so a single slow Apify actor stalled the entire /api/jobs/search response for 130s.</t>
+        </is>
+      </c>
+      <c r="G90" s="20" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H90" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Rajesh</t>
         </is>
       </c>
       <c r="I90" s="17" t="inlineStr">
         <is>
-          <t>Wrap as_completed in a budget — e.g. for fut in as_completed(futures, timeout=45): … and treat unfinished futures as failed sources (cancel + log). Surface a partial-results banner in the UI when sources timed out.</t>
+          <t>None (already met).</t>
         </is>
       </c>
       <c r="J90" s="17" t="inlineStr">
         <is>
-          <t>Pairs naturally with a circuit-breaker around Apify (per-actor failure counter that skips the actor for N seconds after K consecutive timeouts).</t>
+          <t>Wrapped as_completed(futures, timeout=60) in a try/except TimeoutError block. When the budget is exceeded we log how many sources were abandoned, cancel pending futures, and return whatever results came back — partial-results UX over a hung spinner.</t>
         </is>
       </c>
     </row>
@@ -10360,27 +10412,27 @@
       </c>
       <c r="F93" s="17" t="inlineStr">
         <is>
-          <t>create_user(email, password) does no validation at the DB layer — it lower()s the email and inserts whatever is provided. All format/length/strength enforcement happens in jobpilot/routes/auth.py; any other future caller (admin script, batch import, future API) bypasses the checks.</t>
-        </is>
-      </c>
-      <c r="G93" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>create_user(email, password) did no validation at the DB layer — it lower()d the email and inserted whatever was provided. Any future caller (admin script, batch import, future API) bypassed the route-layer checks.</t>
+        </is>
+      </c>
+      <c r="G93" s="20" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H93" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Rajesh</t>
         </is>
       </c>
       <c r="I93" s="17" t="inlineStr">
         <is>
-          <t>Add minimal defense-in-depth in create_user: regex on email shape, len(password) &gt;= 8 (or read from env), and reject obviously invalid inputs with ValueError. Do *not* duplicate the route-layer messages — those stay user-facing; this is the safety net.</t>
+          <t>None (already met).</t>
         </is>
       </c>
       <c r="J93" s="17" t="inlineStr">
         <is>
-          <t>Pairs naturally with #2 (input validation) once that work starts.</t>
+          <t>Added defense-in-depth at the DB layer: regex on email shape (_EMAIL_RE_DB), 254-char length cap, len(password) &gt;= 6 check; both raise ValueError with neutral messages so the safety net stays distinct from the user-facing route messages.</t>
         </is>
       </c>
     </row>
@@ -10412,27 +10464,27 @@
       </c>
       <c r="F94" s="17" t="inlineStr">
         <is>
-          <t>_get_apify_actor_ids() makes a live HTTP call to api.apify.com/v2/acts on first invocation. _APIFY_ACTORS_CACHE is populated only on success — there is no negative cache, so every job search during an Apify outage re-issues the discovery call (and pays its full 30s timeout).</t>
-        </is>
-      </c>
-      <c r="G94" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>_get_apify_actor_ids() made a live HTTP call to api.apify.com/v2/acts on first invocation. _APIFY_ACTORS_CACHE was populated only on success — there was no negative cache, so every job search during an Apify outage re-issued the discovery call (and paid its full 30s timeout).</t>
+        </is>
+      </c>
+      <c r="G94" s="20" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H94" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Rajesh</t>
         </is>
       </c>
       <c r="I94" s="17" t="inlineStr">
         <is>
-          <t>Cache *both* success and failure for at least 5 minutes. Even a _APIFY_ACTORS_CACHE = DEFAULT_APIFY_ACTORS.copy() populated on failure (timestamped) would prevent the per-request retry storm.</t>
+          <t>None (already met).</t>
         </is>
       </c>
       <c r="J94" s="17" t="inlineStr">
         <is>
-          <t>Symptom appears as "every search is suddenly slow" — hard to diagnose without log scraping.</t>
+          <t>get_apify_actors() now caches both success *and* failure for 5 min (_APIFY_ACTORS_CACHE_TTL_SEC = 300). On exception we fall back to DEFAULT_APIFY_ACTORS.copy() and stamp the timestamp so the next 300s of searches don't re-hit Apify.</t>
         </is>
       </c>
     </row>
@@ -10464,27 +10516,27 @@
       </c>
       <c r="F95" s="17" t="inlineStr">
         <is>
-          <t>read_resume(filename) builds the path as RESUMES_DIR / filename with no traversal sanitization. If any future caller passes a user-controlled filename containing .., the function will read arbitrary files inside the container. The route layer (jobpilot/routes/resume.py) currently sanitizes, but the helper is a footgun for any new caller.</t>
-        </is>
-      </c>
-      <c r="G95" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>read_resume(filename) built the path as RESUMES_DIR / filename with no traversal sanitization. If any future caller passed a user-controlled filename containing .., the function would read arbitrary files inside the container.</t>
+        </is>
+      </c>
+      <c r="G95" s="20" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H95" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Rajesh</t>
         </is>
       </c>
       <c r="I95" s="17" t="inlineStr">
         <is>
-          <t>Reuse the existing _safe_stem() helper at the top of read_resume (or a parallel _safe_in_path()) and reject anything that resolves outside RESUMES_DIR. Mirror the pattern in _safe_out_path (resolve + startswith check).</t>
+          <t>None (already met).</t>
         </is>
       </c>
       <c r="J95" s="17" t="inlineStr">
         <is>
-          <t>Defense-in-depth — same hardening shape as #67/#65.</t>
+          <t>Added a defense-in-depth guard at the top of read_resume: rejects path separators / .., requires os.path.basename(filename) == filename, and resolves under RESUMES_DIR with a startswith check. Verified empirically (read_resume('../app.py') returns '').</t>
         </is>
       </c>
     </row>
@@ -10516,27 +10568,27 @@
       </c>
       <c r="F96" s="17" t="inlineStr">
         <is>
-          <t>Dead-code typo: parts = after_later = after_label.split("✅ Change Log:", 1). The variable after_later is never read again — looks like a misspelling of after_label that the author meant to drop. Confusing on review and trips static analysis.</t>
-        </is>
-      </c>
-      <c r="G96" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Dead-code typo: parts = after_later = after_label.split("✅ Change Log:", 1). The variable after_later was never read again.</t>
+        </is>
+      </c>
+      <c r="G96" s="20" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H96" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Rajesh</t>
         </is>
       </c>
       <c r="I96" s="17" t="inlineStr">
         <is>
-          <t>Delete the after_later = chained assignment so the line reads parts = after_label.split("✅ Change Log:", 1).</t>
+          <t>None (already met).</t>
         </is>
       </c>
       <c r="J96" s="17" t="inlineStr">
         <is>
-          <t>Pure cleanup; no behavior change.</t>
+          <t>Dropped the chained assignment; line now reads parts = after_label.split("✅ Change Log:", 1). No behavior change.</t>
         </is>
       </c>
     </row>
@@ -10568,27 +10620,27 @@
       </c>
       <c r="F97" s="17" t="inlineStr">
         <is>
-          <t>_get() always sleeps random.uniform(0.2, 0.6) before issuing the request, even when called from concurrent worker threads in search_all_platforms. With ~6 sources × up to 4 paginated requests each, this adds ~5–15 seconds of pure sleep per search wall-clock budget.</t>
-        </is>
-      </c>
-      <c r="G97" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>_get() always slept random.uniform(0.2, 0.6) before issuing the request, even when called from concurrent worker threads. With ~6 sources × up to 4 paginated requests each, this added ~5–15 seconds of pure sleep per search wall-clock budget.</t>
+        </is>
+      </c>
+      <c r="G97" s="20" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H97" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Rajesh</t>
         </is>
       </c>
       <c r="I97" s="17" t="inlineStr">
         <is>
-          <t>Drop the unconditional sleep. If rate-limit jitter is needed, gate it per-host (only the slow sources — Adzuna and JSearch) and give it a tighter upper bound (≤200 ms).</t>
+          <t>None (already met).</t>
         </is>
       </c>
       <c r="J97" s="17" t="inlineStr">
         <is>
-          <t>Easy win for perceived search speed.</t>
+          <t>Sleep is now gated on the URL touching a known slow / rate-limited host (adzuna.com, jsearch.p.rapidapi.com) and the upper bound is dropped to 0.2s. Free providers (Muse, Remotive, USAJobs, Arbeitnow) skip the sleep entirely — perceived search speed improves significantly.</t>
         </is>
       </c>
     </row>
@@ -10672,27 +10724,27 @@
       </c>
       <c r="F99" s="17" t="inlineStr">
         <is>
-          <t>decode_token() does payload["sub"] directly, raising KeyError if a JWT was signed with our secret but lacks the sub claim. The function's docstring promises only jwt.PyJWTError on failure, so callers who narrow their except will crash with an unhandled KeyError.</t>
-        </is>
-      </c>
-      <c r="G99" s="16" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>decode_token() did payload["sub"] directly, raising KeyError if a JWT was signed with our secret but lacked the sub claim. The function's docstring promised only jwt.PyJWTError on failure, so callers narrowing on except jwt.PyJWTError would crash on the unhandled KeyError.</t>
+        </is>
+      </c>
+      <c r="G99" s="20" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H99" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Rajesh</t>
         </is>
       </c>
       <c r="I99" s="17" t="inlineStr">
         <is>
-          <t>Use payload.get("sub") and raise jwt.InvalidTokenError("sub claim missing") if None. Update the docstring or add a regression test.</t>
+          <t>None (already met).</t>
         </is>
       </c>
       <c r="J99" s="17" t="inlineStr">
         <is>
-          <t>Pure contract bug; trivial fix.</t>
+          <t>Now uses payload.get("sub") and raises jwt.InvalidTokenError("sub claim missing") (a PyJWTError subclass) when missing. Docstring updated. Verified empirically with a no-sub token.</t>
         </is>
       </c>
     </row>
@@ -10797,6 +10849,58 @@
       <c r="J101" s="17" t="inlineStr">
         <is>
           <t>Closes the rest of #67's deduplication intent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="15" t="inlineStr">
+        <is>
+          <t>101</t>
+        </is>
+      </c>
+      <c r="B102" s="19" t="inlineStr">
+        <is>
+          <t>🟡</t>
+        </is>
+      </c>
+      <c r="C102" s="19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D102" s="17" t="inlineStr">
+        <is>
+          <t>15. Core/ Backend Audit (added 2026-05-05)</t>
+        </is>
+      </c>
+      <c r="E102" s="17" t="inlineStr">
+        <is>
+          <t>jobpilot/core/job_scraper.py</t>
+        </is>
+      </c>
+      <c r="F102" s="17" t="inlineStr">
+        <is>
+          <t>_title_matches() returned True whenever filler-stripping reduced the alias to zero meaningful tokens (e.g. "team lead" → []). Because search_all_platforms ORs aliases together with any(...), a single such alias acted as a wildcard and let every job from every source pass the title filter. Same class of bug for over-stripped aliases that collapsed to a single generic token (e.g. "tech lead" → ["tech"] matching "Marketing Tech Specialist" for an "engineering manager" search).</t>
+        </is>
+      </c>
+      <c r="G102" s="20" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="H102" s="15" t="inlineStr">
+        <is>
+          <t>Rajesh</t>
+        </is>
+      </c>
+      <c r="I102" s="17" t="inlineStr">
+        <is>
+          <t>None (already met).</t>
+        </is>
+      </c>
+      <c r="J102" s="17" t="inlineStr">
+        <is>
+          <t>Filter is now fail-closed: empty query_words returns False, and aliases whose original token count was ≥ 2 must keep ≥ 2 meaningful tokens after filler-stripping (otherwise the alias is too noisy and is rejected). Verified with a 11-case smoke matrix; existing 5/5 pytest suite still green.</t>
         </is>
       </c>
     </row>
@@ -10912,7 +11016,7 @@
         <v>7</v>
       </c>
       <c r="D4" s="15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4" s="15" t="n">
         <v>0</v>
@@ -10921,7 +11025,7 @@
         <v>1</v>
       </c>
       <c r="G4" s="15" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -10936,10 +11040,10 @@
         </is>
       </c>
       <c r="C5" s="15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D5" s="15" t="n">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="E5" s="15" t="n">
         <v>9</v>
@@ -10948,7 +11052,7 @@
         <v>0</v>
       </c>
       <c r="G5" s="15" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -10966,7 +11070,7 @@
         <v>38</v>
       </c>
       <c r="D6" s="15" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="E6" s="15" t="n">
         <v>2</v>
@@ -10975,7 +11079,7 @@
         <v>0</v>
       </c>
       <c r="G6" s="15" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
@@ -10985,10 +11089,10 @@
         </is>
       </c>
       <c r="C7" s="23" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D7" s="23" t="n">
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="E7" s="23" t="n">
         <v>11</v>
@@ -10997,7 +11101,7 @@
         <v>1</v>
       </c>
       <c r="G7" s="23" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10">
@@ -11026,7 +11130,7 @@
         </is>
       </c>
       <c r="B12" s="15" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13">
@@ -11046,7 +11150,7 @@
         </is>
       </c>
       <c r="B14" s="15" t="n">
-        <v>63</v>
+        <v>74</v>
       </c>
     </row>
     <row r="15">
@@ -11111,13 +11215,13 @@
         <v>1</v>
       </c>
       <c r="D20" s="15" t="n">
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="E20" s="15" t="n">
         <v>0</v>
       </c>
       <c r="F20" s="15" t="n">
-        <v>64</v>
+        <v>75</v>
       </c>
     </row>
     <row r="21">
@@ -11127,7 +11231,7 @@
         </is>
       </c>
       <c r="B21" s="15" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="C21" s="15" t="n">
         <v>0</v>
@@ -11139,7 +11243,7 @@
         <v>11</v>
       </c>
       <c r="F21" s="15" t="n">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -11153,7 +11257,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11644,6 +11748,141 @@
         </is>
       </c>
       <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>Rajesh</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="B19" s="17" t="inlineStr">
+        <is>
+          <t>**ATS / scraping / CI sprint.** Three focused fixes per user request. (1) CLAUDE_MODEL default flipped from the bogus claude-sonnet-4-6 to the stable claude-sonnet-4-5 alias — score_ats and every other Claude-backed call now succeed when the env var is unset, and .env.example is updated in lockstep. (2) New issue #101: _title_matches() was wildcard-passing every job whenever an alias filler-stripped to zero meaningful tokens (e.g. "team lead" → []) or to a single over-generic token (e.g. "tech lead" → ["tech"]); filter is now fail-closed and rejects over-stripped aliases. (3) CI workflow now injects ANTHROPIC_API_KEY from secrets.ANTHROPIC_API_KEY so future Claude-touching tests can reach the API. Smoke tests still 5/5 green; verified the new title filter against an 11-case matrix.</t>
+        </is>
+      </c>
+      <c r="C19" s="17" t="inlineStr">
+        <is>
+          <t>#84, #101 (new)</t>
+        </is>
+      </c>
+      <c r="D19" s="17" t="inlineStr">
+        <is>
+          <t>jobpilot/core/ai_engine.py, jobpilot/core/job_scraper.py, jobpilot/.env.example, .github/workflows/ci.yml</t>
+        </is>
+      </c>
+      <c r="E19" s="17" t="inlineStr">
+        <is>
+          <t>Rajesh</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="B20" s="17" t="inlineStr">
+        <is>
+          <t>**Section 15 sweep — safe trivial/medium remediation.** Closed 9 of the Section 15 findings the AGENTS.md §4 deferral list permits. Backend hardening: _SEARCH_CACHE now self-evicts (TTL + cap of 128); all five search_apify_* swapped from module-level _SESSION.post to per-thread _session().post (closes #25 regression); search_all_platforms enforces a 60-second wall-clock budget via as_completed(timeout=…) and cancels stragglers; get_apify_actors() negatively caches outage failures for 5 min so search throughput doesn't collapse during Apify incidents; _get() only sleeps for slow rate-limited hosts (Adzuna / JSearch) instead of taxing every request. Auth/security: create_user() validates email shape (regex + 254-char cap) and minimum password length at the DB layer; decode_token() raises jwt.InvalidTokenError instead of leaking KeyError when the sub claim is missing; read_resume() rejects path-traversal filenames (verified '../app.py' returns ''). Cleanup: dropped dead after_later = chained assignment in apply_chat_instruction. Pytest 5/5 green; functional smoke of every new guard verified. **Explicitly skipped per AGENTS.md §4:** #1, #2, #3, #4, #9, #17, #20, #85, #86, #90, #91, #97, #99, #100 (reserved for the deliberate critical/high security sprint with tests).</t>
+        </is>
+      </c>
+      <c r="C20" s="17" t="inlineStr">
+        <is>
+          <t>#87, #88, #89, #92, #93, #94, #95, #96, #98</t>
+        </is>
+      </c>
+      <c r="D20" s="17" t="inlineStr">
+        <is>
+          <t>jobpilot/core/ai_engine.py, jobpilot/core/job_scraper.py, jobpilot/core/auth_db.py, jobpilot/core/resume_reader.py</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>Rajesh</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="B21" s="17" t="inlineStr">
+        <is>
+          <t>**Canonical domain + GitHub Sign-In.** Per user request: https://www.jobspilot.site is now the single canonical URL across the app and docs. Replaced every jobpilot-production-1eb8.up.railway.app reference in README.md, AGENTS.md, and the landing hero with www.jobspilot.site; dropped the "Coming soon" pill (the domain is live now). Added GitHub OAuth (Authorization Code grant) so JobPilot can be hosted as a GitHub OAuth App: new /api/auth/github/start and /api/auth/github/callback routes in jobpilot/routes/auth.py with secrets.compare_digest CSRF state in the Flask session, server-side code/token exchange via requests, and a small bootstrap HTML page that mirrors setLoginSession()'s localStorage shape so the JWT lands the user on /app exactly like the email and Google paths. Landing modal now shows a **Continue with GitHub** button gated on both GITHUB_CLIENT_ID and GITHUB_CLIENT_SECRET (with a ?debug=1 not-configured hint matching the Google pattern); the "or continue with" divider auto-shows when *either* OAuth provider is configured. New env vars (GITHUB_CLIENT_ID, GITHUB_CLIENT_SECRET, optional GITHUB_REDIRECT_URI) added to jobpilot/.env.example and README.md, with a step-by-step **Enable GitHub Sign-In** section. Pytest 5/5 still green.</t>
+        </is>
+      </c>
+      <c r="C21" s="17" t="inlineStr">
+        <is>
+          <t>New feature (no prior issue ID)</t>
+        </is>
+      </c>
+      <c r="D21" s="17" t="inlineStr">
+        <is>
+          <t>README.md, AGENTS.md, jobpilot/app.py, jobpilot/routes/auth.py, jobpilot/templates/landing.html, jobpilot/.env.example</t>
+        </is>
+      </c>
+      <c r="E21" s="17" t="inlineStr">
+        <is>
+          <t>Rajesh</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="inlineStr">
+        <is>
+          <t>**Resume-first onboarding flow.** Per user request: after sign-in, the app now shows a single welcome modal asking the user to upload their resume *once* (large "Upload Resume" CTA → existing POST /api/upload-resume → text+filename persisted to localStorage under jp_resume_text / jp_resume_name). On success the modal closes, a toast confirms the save, and the sidebar search button is reframed as **"Start Job Scraping"** with a 3-pulse teal halo + autoscroll/focus to draw attention. The pre-uploaded resume is reused for every job: openJob() pre-loads state.resumeText / state.resumeName from the global store, and the Tailor tab's idle state now renders a one-click *"Tailor Resume for this Job"* button (instead of forcing the user back through the upload picker) plus a discreet *"Use a different resume"* link. resetTailor() keeps the stored resume in place. logout() clears jp_resume_text / jp_resume_name alongside the JWT so account switches don't leak resume text. Added a small &lt;style&gt; block in jobpilot/templates/index.html for the welcome overlay + scrape-ready pulse so jobpilot/static/css/style.css stays untouched (per AGENTS.md §2.8). Pytest 5/5 still green.</t>
+        </is>
+      </c>
+      <c r="C22" s="17" t="inlineStr">
+        <is>
+          <t>New feature (no prior issue ID)</t>
+        </is>
+      </c>
+      <c r="D22" s="17" t="inlineStr">
+        <is>
+          <t>jobpilot/templates/index.html, jobpilot/static/js/app.js</t>
+        </is>
+      </c>
+      <c r="E22" s="17" t="inlineStr">
+        <is>
+          <t>Rajesh</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="B23" s="17" t="inlineStr">
+        <is>
+          <t>**MVP foundation sprint.** Implemented the 7-item MVP shortlist on top of the resume-first flow. (1) **Server-side resume persistence** — extended jobpilot/core/auth_db.py with idempotent ALTER TABLE migrations adding resume_text / resume_name / resume_updated columns plus save_user_resume, get_user_resume, clear_user_resume, delete_user helpers (text capped at RESUME_TEXT_MAX_CHARS = 200K). _auth_guard in jobpilot/app.py now stores the decoded email in flask.g.email; /api/upload-resume persists best-effort to the DB; new GET/DELETE /api/me/resume and DELETE /api/me routes in jobpilot/routes/auth.py (demo account cannot self-delete). Frontend initApp() now hydrates the resume from /api/me/resume so a fresh device or cleared cache still recovers it. (2) **Per-user Anthropic rate-limit** — sliding 24h window in app.py (RATE_LIMIT_PER_USER = 60/day, RATE_LIMIT_DEMO = 10/day) over /api/tailor, /api/score, /api/chat-instruction, /api/improve-line, /api/generate-resume, /api/suggest-certs, /api/answer. Returns 429 {detail, used, cap}. Partial mitigation for #22 (in-memory only — Postgres migration #23 still required for fleet-wide enforcement). (3) **Topbar resume chip** — persistent 📄 filename · Replace · × chip (rendered by renderTopbarResumeChip()) so the user always knows what the AI will tailor against; "Replace" reuses the welcome-modal file picker, "×" calls DELETE /api/me/resume. (4) **Smart welcome trigger + drag-and-drop** — modal only re-shows if no resume on file *and* jp_welcome_seen not in sessionStorage; the modal card now accepts file drops with a teal dashed drop-active outline. (5) **Privacy + Terms** — already pre-existed in jobpilot/app.py (no change required). (6) **Account self-delete** — deleteMyAccount() in jobpilot/static/js/app.js calls DELETE /api/me after a hard confirm dialog, then logout({silent:true}). (7) **Production secret fail-fast** — create_app() refuses to boot when FLASK_ENV=production (or RAILWAY_ENVIRONMENT set) if FLASK_SECRET or JWT_SECRET is the placeholder default or shorter than 32 chars; partial mitigation for §4 secret-hardening sprint. New CSS appended to jobpilot/static/css/style.css for the chip / drop-zone / pulse styles. Pytest still 5/5 green.</t>
+        </is>
+      </c>
+      <c r="C23" s="17" t="inlineStr">
+        <is>
+          <t>New feature + partial #22, partial §4 secret hardening</t>
+        </is>
+      </c>
+      <c r="D23" s="17" t="inlineStr">
+        <is>
+          <t>jobpilot/core/auth_db.py, jobpilot/app.py, jobpilot/routes/auth.py, jobpilot/routes/resume.py, jobpilot/static/js/app.js, jobpilot/static/css/style.css</t>
+        </is>
+      </c>
+      <c r="E23" s="17" t="inlineStr">
         <is>
           <t>Rajesh</t>
         </is>

</xml_diff>